<commit_message>
Switched to KINEC v3 database.
</commit_message>
<xml_diff>
--- a/Projects/Vulkaneifel/Data_Sheet_Vulkaneifel.xlsx
+++ b/Projects/Vulkaneifel/Data_Sheet_Vulkaneifel.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TamaraMichaelis\Code\SMEW\Projects\Vulkaneifel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0B5AEF5-0488-4599-BDF4-0435BF06779B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91122E12-36A3-4D4C-A3C1-BF16D648CA24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="760" yWindow="760" windowWidth="14400" windowHeight="7270" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Climatic" sheetId="1" r:id="rId1"/>
@@ -341,7 +341,7 @@
     <t>Field C</t>
   </si>
   <si>
-    <t>apatite</t>
+    <t>hydroxyapatite</t>
   </si>
 </sst>
 </file>
@@ -718,7 +718,7 @@
         <v>73</v>
       </c>
       <c r="D2">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
@@ -1360,7 +1360,7 @@
         <v>12</v>
       </c>
       <c r="D4">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="E4" t="s">
         <v>91</v>

</xml_diff>